<commit_message>
Caso 13 Industria: cambia a produccion por lote y retira modelo de paradas de maquina
</commit_message>
<xml_diff>
--- a/PMD1_15_Casos_Sinteticos/13_Industria_PMD1.xlsx
+++ b/PMD1_15_Casos_Sinteticos/13_Industria_PMD1.xlsx
@@ -466,7 +466,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Una fila de Operaciones representa parada de maquina</t>
+          <t>Una fila de Operaciones representa un lote producido en planta</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>En Industria, precio_referencia_soles es el costo referencial por hora de un tipo de parada; el costo real de cada parada varía con la duración y el personal afectado.</t>
+          <t>En Industria, costo_unitario_referencia_soles es el costo estándar por unidad de cada producto; el costo real de cada lote varía con las unidades producidas, los operarios asignados y la antigüedad de la máquina.</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>En Industria, operarios_afectados es el número de operarios detenidos por la parada y costo_parada_soles es el costo total de la parada.</t>
+          <t>En Industria, unidades_producidas es la cantidad de unidades fabricadas en el lote, operarios_asignados es el número de operarios de la línea y costo_lote_soles es el costo total de producción del lote.</t>
         </is>
       </c>
     </row>
@@ -655,12 +655,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>duracion_parada_min</t>
+          <t>unidades_producidas</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>operarios_afectados</t>
+          <t>operarios_asignados</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>costo_parada_soles</t>
+          <t>costo_lote_soles</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>59</v>
+        <v>2360</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
@@ -740,7 +740,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>6</v>
+        <v>240</v>
       </c>
       <c r="G3" t="n">
         <v>1</v>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>27</v>
+        <v>1080</v>
       </c>
       <c r="G4" t="n">
         <v>5</v>
@@ -818,7 +818,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>99</v>
+        <v>3960</v>
       </c>
       <c r="H5" t="n">
         <v>19</v>
@@ -854,7 +854,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>104</v>
+        <v>4160</v>
       </c>
       <c r="G6" t="n">
         <v>6</v>
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>46</v>
+        <v>1840</v>
       </c>
       <c r="G7" t="n">
         <v>5</v>
@@ -932,7 +932,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5</v>
+        <v>200</v>
       </c>
       <c r="G8" t="n">
         <v>1</v>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>46</v>
+        <v>1840</v>
       </c>
       <c r="G9" t="n">
         <v>3</v>
@@ -1010,7 +1010,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>39</v>
+        <v>1560</v>
       </c>
       <c r="G10" t="n">
         <v>3</v>
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>20</v>
+        <v>800</v>
       </c>
       <c r="G11" t="n">
         <v>4</v>
@@ -1088,7 +1088,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>41</v>
+        <v>1640</v>
       </c>
       <c r="G12" t="n">
         <v>4</v>
@@ -1127,7 +1127,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>32</v>
+        <v>1280</v>
       </c>
       <c r="G13" t="n">
         <v>4</v>
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>15</v>
+        <v>600</v>
       </c>
       <c r="G14" t="n">
         <v>1</v>
@@ -1205,7 +1205,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>41</v>
+        <v>1640</v>
       </c>
       <c r="G15" t="n">
         <v>7</v>
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>2640</v>
       </c>
       <c r="G16" t="n">
         <v>3</v>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>35</v>
+        <v>1400</v>
       </c>
       <c r="G17" t="n">
         <v>4</v>
@@ -1322,7 +1322,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>105</v>
+        <v>4200</v>
       </c>
       <c r="G18" t="n">
         <v>7</v>
@@ -1361,7 +1361,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>69</v>
+        <v>2760</v>
       </c>
       <c r="G19" t="n">
         <v>9</v>
@@ -1400,7 +1400,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>88</v>
+        <v>3520</v>
       </c>
       <c r="G20" t="n">
         <v>9</v>
@@ -1439,7 +1439,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>42</v>
+        <v>1680</v>
       </c>
       <c r="G21" t="n">
         <v>4</v>
@@ -1478,7 +1478,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>72</v>
+        <v>2880</v>
       </c>
       <c r="G22" t="n">
         <v>3</v>
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>77</v>
+        <v>3080</v>
       </c>
       <c r="G23" t="n">
         <v>7</v>
@@ -1556,7 +1556,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>85</v>
+        <v>3400</v>
       </c>
       <c r="G24" t="n">
         <v>4</v>
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>70</v>
+        <v>2800</v>
       </c>
       <c r="G25" t="n">
         <v>9</v>
@@ -1634,7 +1634,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>65</v>
+        <v>2600</v>
       </c>
       <c r="G26" t="n">
         <v>4</v>
@@ -1673,7 +1673,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>36</v>
+        <v>1440</v>
       </c>
       <c r="G27" t="n">
         <v>1</v>
@@ -1712,7 +1712,7 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>55</v>
+        <v>2200</v>
       </c>
       <c r="G28" t="n">
         <v>5</v>
@@ -1751,7 +1751,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>9</v>
+        <v>360</v>
       </c>
       <c r="G29" t="n">
         <v>2</v>
@@ -1790,7 +1790,7 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>121</v>
+        <v>4840</v>
       </c>
       <c r="G30" t="n">
         <v>9</v>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>50</v>
+        <v>2000</v>
       </c>
       <c r="G31" t="n">
         <v>2</v>
@@ -1868,7 +1868,7 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>35</v>
+        <v>1400</v>
       </c>
       <c r="G32" t="n">
         <v>3</v>
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>20</v>
+        <v>800</v>
       </c>
       <c r="G33" t="n">
         <v>4</v>
@@ -1946,7 +1946,7 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>38</v>
+        <v>1520</v>
       </c>
       <c r="G34" t="n">
         <v>1</v>
@@ -1985,7 +1985,7 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>33</v>
+        <v>1320</v>
       </c>
       <c r="G35" t="n">
         <v>2</v>
@@ -2024,7 +2024,7 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>107</v>
+        <v>4280</v>
       </c>
       <c r="G36" t="n">
         <v>7</v>
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>20</v>
+        <v>800</v>
       </c>
       <c r="G37" t="n">
         <v>3</v>
@@ -2102,7 +2102,7 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>66</v>
+        <v>2640</v>
       </c>
       <c r="G38" t="n">
         <v>3</v>
@@ -2141,7 +2141,7 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>31</v>
+        <v>1240</v>
       </c>
       <c r="G39" t="n">
         <v>4</v>
@@ -2180,7 +2180,7 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>60</v>
+        <v>2400</v>
       </c>
       <c r="G40" t="n">
         <v>6</v>
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>22</v>
+        <v>880</v>
       </c>
       <c r="G41" t="n">
         <v>1</v>
@@ -2258,7 +2258,7 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>5</v>
+        <v>200</v>
       </c>
       <c r="G42" t="n">
         <v>2</v>
@@ -2297,7 +2297,7 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>52</v>
+        <v>2080</v>
       </c>
       <c r="G43" t="n">
         <v>3</v>
@@ -2336,7 +2336,7 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>32</v>
+        <v>1280</v>
       </c>
       <c r="G44" t="n">
         <v>2</v>
@@ -2375,7 +2375,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>8</v>
+        <v>320</v>
       </c>
       <c r="H45" t="n">
         <v>20</v>
@@ -2411,7 +2411,7 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>33</v>
+        <v>1320</v>
       </c>
       <c r="G46" t="n">
         <v>1</v>
@@ -2450,7 +2450,7 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>7</v>
+        <v>280</v>
       </c>
       <c r="G47" t="n">
         <v>1</v>
@@ -2489,7 +2489,7 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>96</v>
+        <v>3840</v>
       </c>
       <c r="G48" t="n">
         <v>6</v>
@@ -2528,7 +2528,7 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>18</v>
+        <v>720</v>
       </c>
       <c r="G49" t="n">
         <v>2</v>
@@ -2567,7 +2567,7 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>42</v>
+        <v>1680</v>
       </c>
       <c r="G50" t="n">
         <v>8</v>
@@ -2606,7 +2606,7 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>46</v>
+        <v>1840</v>
       </c>
       <c r="G51" t="n">
         <v>3</v>
@@ -2645,7 +2645,7 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>51</v>
+        <v>2040</v>
       </c>
       <c r="G52" t="n">
         <v>3</v>
@@ -2684,7 +2684,7 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>54</v>
+        <v>2160</v>
       </c>
       <c r="G53" t="n">
         <v>4</v>
@@ -2723,7 +2723,7 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>80</v>
+        <v>3200</v>
       </c>
       <c r="G54" t="n">
         <v>6</v>
@@ -2762,7 +2762,7 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>46</v>
+        <v>1840</v>
       </c>
       <c r="G55" t="n">
         <v>4</v>
@@ -2801,7 +2801,7 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>98</v>
+        <v>3920</v>
       </c>
       <c r="G56" t="n">
         <v>7</v>
@@ -2840,7 +2840,7 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>26</v>
+        <v>1040</v>
       </c>
       <c r="G57" t="n">
         <v>3</v>
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>89</v>
+        <v>3560</v>
       </c>
       <c r="G58" t="n">
         <v>6</v>
@@ -2918,7 +2918,7 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>67</v>
+        <v>2680</v>
       </c>
       <c r="G59" t="n">
         <v>2</v>
@@ -2957,7 +2957,7 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>61</v>
+        <v>2440</v>
       </c>
       <c r="G60" t="n">
         <v>6</v>
@@ -2996,7 +2996,7 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>40</v>
+        <v>1600</v>
       </c>
       <c r="G61" t="n">
         <v>7</v>
@@ -3035,7 +3035,7 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>16</v>
+        <v>640</v>
       </c>
       <c r="G62" t="n">
         <v>2</v>
@@ -3074,7 +3074,7 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>51</v>
+        <v>2040</v>
       </c>
       <c r="G63" t="n">
         <v>3</v>
@@ -3113,7 +3113,7 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>69</v>
+        <v>2760</v>
       </c>
       <c r="G64" t="n">
         <v>3</v>
@@ -3152,7 +3152,7 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>28</v>
+        <v>1120</v>
       </c>
       <c r="G65" t="n">
         <v>2</v>
@@ -3191,7 +3191,7 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>19</v>
+        <v>760</v>
       </c>
       <c r="G66" t="n">
         <v>1</v>
@@ -3230,7 +3230,7 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>50</v>
+        <v>2000</v>
       </c>
       <c r="G67" t="n">
         <v>5</v>
@@ -3269,7 +3269,7 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>59</v>
+        <v>2360</v>
       </c>
       <c r="G68" t="n">
         <v>4</v>
@@ -3308,7 +3308,7 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>58</v>
+        <v>2320</v>
       </c>
       <c r="G69" t="n">
         <v>4</v>
@@ -3347,7 +3347,7 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>102</v>
+        <v>4080</v>
       </c>
       <c r="G70" t="n">
         <v>9</v>
@@ -3386,7 +3386,7 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>90</v>
+        <v>3600</v>
       </c>
       <c r="G71" t="n">
         <v>7</v>
@@ -3425,7 +3425,7 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>66</v>
+        <v>2640</v>
       </c>
       <c r="G72" t="n">
         <v>4</v>
@@ -3464,7 +3464,7 @@
         </is>
       </c>
       <c r="F73" t="n">
-        <v>35</v>
+        <v>1400</v>
       </c>
       <c r="G73" t="n">
         <v>5</v>
@@ -3503,7 +3503,7 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>72</v>
+        <v>2880</v>
       </c>
       <c r="G74" t="n">
         <v>5</v>
@@ -3542,7 +3542,7 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>18</v>
+        <v>720</v>
       </c>
       <c r="H75" t="n">
         <v>22</v>
@@ -3578,7 +3578,7 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>116</v>
+        <v>4640</v>
       </c>
       <c r="G76" t="n">
         <v>9</v>
@@ -3617,7 +3617,7 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>50</v>
+        <v>2000</v>
       </c>
       <c r="G77" t="n">
         <v>5</v>
@@ -3656,7 +3656,7 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>68</v>
+        <v>2720</v>
       </c>
       <c r="G78" t="n">
         <v>2</v>
@@ -3695,7 +3695,7 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>76</v>
+        <v>3040</v>
       </c>
       <c r="G79" t="n">
         <v>4</v>
@@ -3734,7 +3734,7 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>52</v>
+        <v>2080</v>
       </c>
       <c r="G80" t="n">
         <v>2</v>
@@ -3773,7 +3773,7 @@
         </is>
       </c>
       <c r="F81" t="n">
-        <v>78</v>
+        <v>3120</v>
       </c>
       <c r="G81" t="n">
         <v>4</v>
@@ -3812,7 +3812,7 @@
         </is>
       </c>
       <c r="F82" t="n">
-        <v>27</v>
+        <v>1080</v>
       </c>
       <c r="G82" t="n">
         <v>2</v>
@@ -3851,7 +3851,7 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>26</v>
+        <v>1040</v>
       </c>
       <c r="G83" t="n">
         <v>4</v>
@@ -3890,7 +3890,7 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>121</v>
+        <v>4840</v>
       </c>
       <c r="G84" t="n">
         <v>11</v>
@@ -3929,7 +3929,7 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>5</v>
+        <v>200</v>
       </c>
       <c r="G85" t="n">
         <v>4</v>
@@ -3968,7 +3968,7 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>74</v>
+        <v>2960</v>
       </c>
       <c r="G86" t="n">
         <v>1</v>
@@ -4007,7 +4007,7 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>31</v>
+        <v>1240</v>
       </c>
       <c r="G87" t="n">
         <v>2</v>
@@ -4046,7 +4046,7 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>81</v>
+        <v>3240</v>
       </c>
       <c r="G88" t="n">
         <v>5</v>
@@ -4085,7 +4085,7 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>19</v>
+        <v>760</v>
       </c>
       <c r="G89" t="n">
         <v>1</v>
@@ -4124,7 +4124,7 @@
         </is>
       </c>
       <c r="F90" t="n">
-        <v>51</v>
+        <v>2040</v>
       </c>
       <c r="G90" t="n">
         <v>3</v>
@@ -4163,7 +4163,7 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>43</v>
+        <v>1720</v>
       </c>
       <c r="G91" t="n">
         <v>3</v>
@@ -4202,7 +4202,7 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>30</v>
+        <v>1200</v>
       </c>
       <c r="G92" t="n">
         <v>2</v>
@@ -4241,7 +4241,7 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>15</v>
+        <v>600</v>
       </c>
       <c r="G93" t="n">
         <v>6</v>
@@ -4280,7 +4280,7 @@
         </is>
       </c>
       <c r="F94" t="n">
-        <v>51</v>
+        <v>2040</v>
       </c>
       <c r="G94" t="n">
         <v>4</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="F95" t="n">
-        <v>74</v>
+        <v>2960</v>
       </c>
       <c r="G95" t="n">
         <v>7</v>
@@ -4358,7 +4358,7 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>45</v>
+        <v>1800</v>
       </c>
       <c r="G96" t="n">
         <v>1</v>
@@ -4397,7 +4397,7 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>55</v>
+        <v>2200</v>
       </c>
       <c r="G97" t="n">
         <v>2</v>
@@ -4436,7 +4436,7 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>67</v>
+        <v>2680</v>
       </c>
       <c r="G98" t="n">
         <v>5</v>
@@ -4475,7 +4475,7 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>62</v>
+        <v>2480</v>
       </c>
       <c r="G99" t="n">
         <v>2</v>
@@ -4511,7 +4511,7 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>71</v>
+        <v>2840</v>
       </c>
       <c r="G100" t="n">
         <v>7</v>
@@ -4550,7 +4550,7 @@
         </is>
       </c>
       <c r="F101" t="n">
-        <v>44</v>
+        <v>1760</v>
       </c>
       <c r="G101" t="n">
         <v>2</v>
@@ -4589,7 +4589,7 @@
         </is>
       </c>
       <c r="F102" t="n">
-        <v>78</v>
+        <v>3120</v>
       </c>
       <c r="G102" t="n">
         <v>2</v>
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="F103" t="n">
-        <v>67</v>
+        <v>2680</v>
       </c>
       <c r="G103" t="n">
         <v>4</v>
@@ -4667,7 +4667,7 @@
         </is>
       </c>
       <c r="F104" t="n">
-        <v>69</v>
+        <v>2760</v>
       </c>
       <c r="G104" t="n">
         <v>9</v>
@@ -4706,7 +4706,7 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>63</v>
+        <v>2520</v>
       </c>
       <c r="G105" t="n">
         <v>8</v>
@@ -4745,7 +4745,7 @@
         </is>
       </c>
       <c r="F106" t="n">
-        <v>68</v>
+        <v>2720</v>
       </c>
       <c r="G106" t="n">
         <v>6</v>
@@ -4784,7 +4784,7 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>108</v>
+        <v>4320</v>
       </c>
       <c r="G107" t="n">
         <v>7</v>
@@ -4823,7 +4823,7 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>75</v>
+        <v>3000</v>
       </c>
       <c r="G108" t="n">
         <v>6</v>
@@ -4862,7 +4862,7 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>81</v>
+        <v>3240</v>
       </c>
       <c r="G109" t="n">
         <v>8</v>
@@ -4901,7 +4901,7 @@
         </is>
       </c>
       <c r="F110" t="n">
-        <v>47</v>
+        <v>1880</v>
       </c>
       <c r="G110" t="n">
         <v>5</v>
@@ -4940,7 +4940,7 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>35</v>
+        <v>1400</v>
       </c>
       <c r="G111" t="n">
         <v>2</v>
@@ -4979,7 +4979,7 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>97</v>
+        <v>3880</v>
       </c>
       <c r="G112" t="n">
         <v>9</v>
@@ -5018,7 +5018,7 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>66</v>
+        <v>2640</v>
       </c>
       <c r="G113" t="n">
         <v>8</v>
@@ -5057,7 +5057,7 @@
         </is>
       </c>
       <c r="F114" t="n">
-        <v>50</v>
+        <v>2000</v>
       </c>
       <c r="G114" t="n">
         <v>5</v>
@@ -5096,7 +5096,7 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>87</v>
+        <v>3480</v>
       </c>
       <c r="G115" t="n">
         <v>7</v>
@@ -5135,7 +5135,7 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>68</v>
+        <v>2720</v>
       </c>
       <c r="G116" t="n">
         <v>4</v>
@@ -5174,7 +5174,7 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>74</v>
+        <v>2960</v>
       </c>
       <c r="G117" t="n">
         <v>5</v>
@@ -5213,7 +5213,7 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>11</v>
+        <v>440</v>
       </c>
       <c r="G118" t="n">
         <v>1</v>
@@ -5252,7 +5252,7 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>42</v>
+        <v>1680</v>
       </c>
       <c r="G119" t="n">
         <v>4</v>
@@ -5291,7 +5291,7 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>42</v>
+        <v>1680</v>
       </c>
       <c r="G120" t="n">
         <v>1</v>
@@ -5330,7 +5330,7 @@
         </is>
       </c>
       <c r="F121" t="n">
-        <v>41</v>
+        <v>1640</v>
       </c>
       <c r="G121" t="n">
         <v>4</v>
@@ -5369,7 +5369,7 @@
         </is>
       </c>
       <c r="F122" t="n">
-        <v>78</v>
+        <v>3120</v>
       </c>
       <c r="G122" t="n">
         <v>6</v>
@@ -5408,7 +5408,7 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>79</v>
+        <v>3160</v>
       </c>
       <c r="G123" t="n">
         <v>9</v>
@@ -5447,7 +5447,7 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>61</v>
+        <v>2440</v>
       </c>
       <c r="G124" t="n">
         <v>2</v>
@@ -5486,7 +5486,7 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>26</v>
+        <v>1040</v>
       </c>
       <c r="G125" t="n">
         <v>3</v>
@@ -5525,7 +5525,7 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>50</v>
+        <v>2000</v>
       </c>
       <c r="G126" t="n">
         <v>6</v>
@@ -5564,7 +5564,7 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>87</v>
+        <v>3480</v>
       </c>
       <c r="G127" t="n">
         <v>6</v>
@@ -5603,7 +5603,7 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>49</v>
+        <v>1960</v>
       </c>
       <c r="G128" t="n">
         <v>4</v>
@@ -5642,7 +5642,7 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>85</v>
+        <v>3400</v>
       </c>
       <c r="G129" t="n">
         <v>7</v>
@@ -5681,7 +5681,7 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>55</v>
+        <v>2200</v>
       </c>
       <c r="G130" t="n">
         <v>3</v>
@@ -5720,7 +5720,7 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>29</v>
+        <v>1160</v>
       </c>
       <c r="G131" t="n">
         <v>3</v>
@@ -5759,7 +5759,7 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>34</v>
+        <v>1360</v>
       </c>
       <c r="G132" t="n">
         <v>4</v>
@@ -5798,7 +5798,7 @@
         </is>
       </c>
       <c r="F133" t="n">
-        <v>19</v>
+        <v>760</v>
       </c>
       <c r="G133" t="n">
         <v>2</v>
@@ -5837,7 +5837,7 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>71</v>
+        <v>2840</v>
       </c>
       <c r="G134" t="n">
         <v>5</v>
@@ -5876,7 +5876,7 @@
         </is>
       </c>
       <c r="F135" t="n">
-        <v>45</v>
+        <v>1800</v>
       </c>
       <c r="G135" t="n">
         <v>3</v>
@@ -5915,7 +5915,7 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>26</v>
+        <v>1040</v>
       </c>
       <c r="G136" t="n">
         <v>4</v>
@@ -5954,7 +5954,7 @@
         </is>
       </c>
       <c r="F137" t="n">
-        <v>98</v>
+        <v>3920</v>
       </c>
       <c r="G137" t="n">
         <v>5</v>
@@ -5993,7 +5993,7 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>75</v>
+        <v>3000</v>
       </c>
       <c r="G138" t="n">
         <v>3</v>
@@ -6032,7 +6032,7 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>56</v>
+        <v>2240</v>
       </c>
       <c r="G139" t="n">
         <v>8</v>
@@ -6107,7 +6107,7 @@
         </is>
       </c>
       <c r="F141" t="n">
-        <v>30</v>
+        <v>1200</v>
       </c>
       <c r="G141" t="n">
         <v>2</v>
@@ -6146,7 +6146,7 @@
         </is>
       </c>
       <c r="F142" t="n">
-        <v>53</v>
+        <v>2120</v>
       </c>
       <c r="G142" t="n">
         <v>9</v>
@@ -6185,7 +6185,7 @@
         </is>
       </c>
       <c r="F143" t="n">
-        <v>11</v>
+        <v>440</v>
       </c>
       <c r="G143" t="n">
         <v>3</v>
@@ -6224,7 +6224,7 @@
         </is>
       </c>
       <c r="F144" t="n">
-        <v>75</v>
+        <v>3000</v>
       </c>
       <c r="G144" t="n">
         <v>5</v>
@@ -6263,7 +6263,7 @@
         </is>
       </c>
       <c r="F145" t="n">
-        <v>84</v>
+        <v>3360</v>
       </c>
       <c r="G145" t="n">
         <v>5</v>
@@ -6302,7 +6302,7 @@
         </is>
       </c>
       <c r="F146" t="n">
-        <v>65</v>
+        <v>2600</v>
       </c>
       <c r="G146" t="n">
         <v>6</v>
@@ -6341,7 +6341,7 @@
         </is>
       </c>
       <c r="F147" t="n">
-        <v>68</v>
+        <v>2720</v>
       </c>
       <c r="G147" t="n">
         <v>9</v>
@@ -6380,7 +6380,7 @@
         </is>
       </c>
       <c r="F148" t="n">
-        <v>37</v>
+        <v>1480</v>
       </c>
       <c r="G148" t="n">
         <v>1</v>
@@ -6419,7 +6419,7 @@
         </is>
       </c>
       <c r="F149" t="n">
-        <v>50</v>
+        <v>2000</v>
       </c>
       <c r="G149" t="n">
         <v>5</v>
@@ -6458,7 +6458,7 @@
         </is>
       </c>
       <c r="F150" t="n">
-        <v>5</v>
+        <v>200</v>
       </c>
       <c r="G150" t="n">
         <v>3</v>
@@ -6497,7 +6497,7 @@
         </is>
       </c>
       <c r="F151" t="n">
-        <v>23</v>
+        <v>920</v>
       </c>
       <c r="G151" t="n">
         <v>2</v>
@@ -6536,7 +6536,7 @@
         </is>
       </c>
       <c r="F152" t="n">
-        <v>59</v>
+        <v>2360</v>
       </c>
       <c r="G152" t="n">
         <v>6</v>
@@ -6575,7 +6575,7 @@
         </is>
       </c>
       <c r="F153" t="n">
-        <v>71</v>
+        <v>2840</v>
       </c>
       <c r="G153" t="n">
         <v>5</v>
@@ -6614,7 +6614,7 @@
         </is>
       </c>
       <c r="F154" t="n">
-        <v>61</v>
+        <v>2440</v>
       </c>
       <c r="G154" t="n">
         <v>7</v>
@@ -6653,7 +6653,7 @@
         </is>
       </c>
       <c r="F155" t="n">
-        <v>63</v>
+        <v>2520</v>
       </c>
       <c r="G155" t="n">
         <v>5</v>
@@ -6692,7 +6692,7 @@
         </is>
       </c>
       <c r="F156" t="n">
-        <v>69</v>
+        <v>2760</v>
       </c>
       <c r="G156" t="n">
         <v>5</v>
@@ -6731,7 +6731,7 @@
         </is>
       </c>
       <c r="F157" t="n">
-        <v>62</v>
+        <v>2480</v>
       </c>
       <c r="G157" t="n">
         <v>3</v>
@@ -6770,7 +6770,7 @@
         </is>
       </c>
       <c r="F158" t="n">
-        <v>57</v>
+        <v>2280</v>
       </c>
       <c r="G158" t="n">
         <v>7</v>
@@ -6809,7 +6809,7 @@
         </is>
       </c>
       <c r="F159" t="n">
-        <v>25</v>
+        <v>1000</v>
       </c>
       <c r="G159" t="n">
         <v>1</v>
@@ -6848,7 +6848,7 @@
         </is>
       </c>
       <c r="F160" t="n">
-        <v>64</v>
+        <v>2560</v>
       </c>
       <c r="G160" t="n">
         <v>6</v>
@@ -6887,7 +6887,7 @@
         </is>
       </c>
       <c r="F161" t="n">
-        <v>105</v>
+        <v>4200</v>
       </c>
       <c r="G161" t="n">
         <v>8</v>
@@ -6926,7 +6926,7 @@
         </is>
       </c>
       <c r="F162" t="n">
-        <v>41</v>
+        <v>1640</v>
       </c>
       <c r="G162" t="n">
         <v>3</v>
@@ -6965,7 +6965,7 @@
         </is>
       </c>
       <c r="F163" t="n">
-        <v>25</v>
+        <v>1000</v>
       </c>
       <c r="G163" t="n">
         <v>6</v>
@@ -7004,7 +7004,7 @@
         </is>
       </c>
       <c r="F164" t="n">
-        <v>89</v>
+        <v>3560</v>
       </c>
       <c r="G164" t="n">
         <v>4</v>
@@ -7043,7 +7043,7 @@
         </is>
       </c>
       <c r="F165" t="n">
-        <v>30</v>
+        <v>1200</v>
       </c>
       <c r="G165" t="n">
         <v>5</v>
@@ -7082,7 +7082,7 @@
         </is>
       </c>
       <c r="F166" t="n">
-        <v>49</v>
+        <v>1960</v>
       </c>
       <c r="G166" t="n">
         <v>6</v>
@@ -7121,7 +7121,7 @@
         </is>
       </c>
       <c r="F167" t="n">
-        <v>80</v>
+        <v>3200</v>
       </c>
       <c r="G167" t="n">
         <v>8</v>
@@ -7160,7 +7160,7 @@
         </is>
       </c>
       <c r="F168" t="n">
-        <v>6</v>
+        <v>240</v>
       </c>
       <c r="G168" t="n">
         <v>1</v>
@@ -7199,7 +7199,7 @@
         </is>
       </c>
       <c r="F169" t="n">
-        <v>26</v>
+        <v>1040</v>
       </c>
       <c r="G169" t="n">
         <v>6</v>
@@ -7238,7 +7238,7 @@
         </is>
       </c>
       <c r="F170" t="n">
-        <v>32</v>
+        <v>1280</v>
       </c>
       <c r="G170" t="n">
         <v>2</v>
@@ -7277,7 +7277,7 @@
         </is>
       </c>
       <c r="F171" t="n">
-        <v>69</v>
+        <v>2760</v>
       </c>
       <c r="G171" t="n">
         <v>3</v>
@@ -7316,7 +7316,7 @@
         </is>
       </c>
       <c r="F172" t="n">
-        <v>28</v>
+        <v>1120</v>
       </c>
       <c r="G172" t="n">
         <v>3</v>
@@ -7355,7 +7355,7 @@
         </is>
       </c>
       <c r="F173" t="n">
-        <v>70</v>
+        <v>2800</v>
       </c>
       <c r="G173" t="n">
         <v>5</v>
@@ -7394,7 +7394,7 @@
         </is>
       </c>
       <c r="F174" t="n">
-        <v>23</v>
+        <v>920</v>
       </c>
       <c r="G174" t="n">
         <v>4</v>
@@ -7433,7 +7433,7 @@
         </is>
       </c>
       <c r="F175" t="n">
-        <v>118</v>
+        <v>4720</v>
       </c>
       <c r="G175" t="n">
         <v>6</v>
@@ -7472,7 +7472,7 @@
         </is>
       </c>
       <c r="F176" t="n">
-        <v>20</v>
+        <v>800</v>
       </c>
       <c r="G176" t="n">
         <v>3</v>
@@ -7511,7 +7511,7 @@
         </is>
       </c>
       <c r="F177" t="n">
-        <v>67</v>
+        <v>2680</v>
       </c>
       <c r="G177" t="n">
         <v>3</v>
@@ -7550,7 +7550,7 @@
         </is>
       </c>
       <c r="F178" t="n">
-        <v>17</v>
+        <v>680</v>
       </c>
       <c r="G178" t="n">
         <v>2</v>
@@ -7589,7 +7589,7 @@
         </is>
       </c>
       <c r="F179" t="n">
-        <v>71</v>
+        <v>2840</v>
       </c>
       <c r="G179" t="n">
         <v>4</v>
@@ -7628,7 +7628,7 @@
         </is>
       </c>
       <c r="F180" t="n">
-        <v>31</v>
+        <v>1240</v>
       </c>
       <c r="G180" t="n">
         <v>5</v>
@@ -7667,7 +7667,7 @@
         </is>
       </c>
       <c r="F181" t="n">
-        <v>6</v>
+        <v>240</v>
       </c>
       <c r="G181" t="n">
         <v>1</v>
@@ -7706,7 +7706,7 @@
         </is>
       </c>
       <c r="F182" t="n">
-        <v>70</v>
+        <v>2800</v>
       </c>
       <c r="G182" t="n">
         <v>6</v>
@@ -7745,7 +7745,7 @@
         </is>
       </c>
       <c r="F183" t="n">
-        <v>65</v>
+        <v>2600</v>
       </c>
       <c r="G183" t="n">
         <v>6</v>
@@ -7784,7 +7784,7 @@
         </is>
       </c>
       <c r="F184" t="n">
-        <v>57</v>
+        <v>2280</v>
       </c>
       <c r="G184" t="n">
         <v>2</v>
@@ -7823,7 +7823,7 @@
         </is>
       </c>
       <c r="F185" t="n">
-        <v>13</v>
+        <v>520</v>
       </c>
       <c r="G185" t="n">
         <v>1</v>
@@ -7862,7 +7862,7 @@
         </is>
       </c>
       <c r="F186" t="n">
-        <v>98</v>
+        <v>3920</v>
       </c>
       <c r="G186" t="n">
         <v>8</v>
@@ -7901,7 +7901,7 @@
         </is>
       </c>
       <c r="F187" t="n">
-        <v>51</v>
+        <v>2040</v>
       </c>
       <c r="G187" t="n">
         <v>1</v>
@@ -7940,7 +7940,7 @@
         </is>
       </c>
       <c r="F188" t="n">
-        <v>51</v>
+        <v>2040</v>
       </c>
       <c r="G188" t="n">
         <v>4</v>
@@ -7979,7 +7979,7 @@
         </is>
       </c>
       <c r="F189" t="n">
-        <v>52</v>
+        <v>2080</v>
       </c>
       <c r="G189" t="n">
         <v>1</v>
@@ -8018,7 +8018,7 @@
         </is>
       </c>
       <c r="F190" t="n">
-        <v>29</v>
+        <v>1160</v>
       </c>
       <c r="G190" t="n">
         <v>5</v>
@@ -8057,7 +8057,7 @@
         </is>
       </c>
       <c r="F191" t="n">
-        <v>59</v>
+        <v>2360</v>
       </c>
       <c r="G191" t="n">
         <v>6</v>
@@ -8096,7 +8096,7 @@
         </is>
       </c>
       <c r="F192" t="n">
-        <v>29</v>
+        <v>1160</v>
       </c>
       <c r="G192" t="n">
         <v>6</v>
@@ -8135,7 +8135,7 @@
         </is>
       </c>
       <c r="F193" t="n">
-        <v>33</v>
+        <v>1320</v>
       </c>
       <c r="G193" t="n">
         <v>2</v>
@@ -8174,7 +8174,7 @@
         </is>
       </c>
       <c r="F194" t="n">
-        <v>59</v>
+        <v>2360</v>
       </c>
       <c r="G194" t="n">
         <v>5</v>
@@ -8213,7 +8213,7 @@
         </is>
       </c>
       <c r="F195" t="n">
-        <v>60</v>
+        <v>2400</v>
       </c>
       <c r="G195" t="n">
         <v>8</v>
@@ -8252,7 +8252,7 @@
         </is>
       </c>
       <c r="F196" t="n">
-        <v>44</v>
+        <v>1760</v>
       </c>
       <c r="G196" t="n">
         <v>5</v>
@@ -8291,7 +8291,7 @@
         </is>
       </c>
       <c r="F197" t="n">
-        <v>71</v>
+        <v>2840</v>
       </c>
       <c r="G197" t="n">
         <v>6</v>
@@ -8330,7 +8330,7 @@
         </is>
       </c>
       <c r="F198" t="n">
-        <v>45</v>
+        <v>1800</v>
       </c>
       <c r="G198" t="n">
         <v>6</v>
@@ -8369,7 +8369,7 @@
         </is>
       </c>
       <c r="F199" t="n">
-        <v>64</v>
+        <v>2560</v>
       </c>
       <c r="G199" t="n">
         <v>5</v>
@@ -8408,7 +8408,7 @@
         </is>
       </c>
       <c r="F200" t="n">
-        <v>94</v>
+        <v>3760</v>
       </c>
       <c r="G200" t="n">
         <v>11</v>
@@ -8447,7 +8447,7 @@
         </is>
       </c>
       <c r="F201" t="n">
-        <v>112</v>
+        <v>4480</v>
       </c>
       <c r="G201" t="n">
         <v>6</v>
@@ -8486,7 +8486,7 @@
         </is>
       </c>
       <c r="F202" t="n">
-        <v>54</v>
+        <v>2160</v>
       </c>
       <c r="G202" t="n">
         <v>5</v>
@@ -8525,7 +8525,7 @@
         </is>
       </c>
       <c r="F203" t="n">
-        <v>11</v>
+        <v>440</v>
       </c>
       <c r="G203" t="n">
         <v>2</v>
@@ -8564,7 +8564,7 @@
         </is>
       </c>
       <c r="F204" t="n">
-        <v>97</v>
+        <v>3880</v>
       </c>
       <c r="G204" t="n">
         <v>10</v>
@@ -8603,7 +8603,7 @@
         </is>
       </c>
       <c r="F205" t="n">
-        <v>23</v>
+        <v>920</v>
       </c>
       <c r="G205" t="n">
         <v>1</v>
@@ -8642,7 +8642,7 @@
         </is>
       </c>
       <c r="F206" t="n">
-        <v>57</v>
+        <v>2280</v>
       </c>
       <c r="G206" t="n">
         <v>1</v>
@@ -8681,7 +8681,7 @@
         </is>
       </c>
       <c r="F207" t="n">
-        <v>59</v>
+        <v>2360</v>
       </c>
       <c r="G207" t="n">
         <v>4</v>
@@ -8720,7 +8720,7 @@
         </is>
       </c>
       <c r="F208" t="n">
-        <v>45</v>
+        <v>1800</v>
       </c>
       <c r="G208" t="n">
         <v>2</v>
@@ -8759,7 +8759,7 @@
         </is>
       </c>
       <c r="F209" t="n">
-        <v>65</v>
+        <v>2600</v>
       </c>
       <c r="G209" t="n">
         <v>6</v>
@@ -8798,7 +8798,7 @@
         </is>
       </c>
       <c r="F210" t="n">
-        <v>33</v>
+        <v>1320</v>
       </c>
       <c r="G210" t="n">
         <v>4</v>
@@ -8837,7 +8837,7 @@
         </is>
       </c>
       <c r="F211" t="n">
-        <v>31</v>
+        <v>1240</v>
       </c>
       <c r="G211" t="n">
         <v>3</v>
@@ -8876,7 +8876,7 @@
         </is>
       </c>
       <c r="F212" t="n">
-        <v>79</v>
+        <v>3160</v>
       </c>
       <c r="G212" t="n">
         <v>5</v>
@@ -8915,7 +8915,7 @@
         </is>
       </c>
       <c r="F213" t="n">
-        <v>34</v>
+        <v>1360</v>
       </c>
       <c r="G213" t="n">
         <v>2</v>
@@ -8954,7 +8954,7 @@
         </is>
       </c>
       <c r="F214" t="n">
-        <v>90</v>
+        <v>3600</v>
       </c>
       <c r="G214" t="n">
         <v>4</v>
@@ -8993,7 +8993,7 @@
         </is>
       </c>
       <c r="F215" t="n">
-        <v>73</v>
+        <v>2920</v>
       </c>
       <c r="G215" t="n">
         <v>5</v>
@@ -9032,7 +9032,7 @@
         </is>
       </c>
       <c r="F216" t="n">
-        <v>39</v>
+        <v>1560</v>
       </c>
       <c r="G216" t="n">
         <v>3</v>
@@ -9071,7 +9071,7 @@
         </is>
       </c>
       <c r="F217" t="n">
-        <v>90</v>
+        <v>3600</v>
       </c>
       <c r="G217" t="n">
         <v>5</v>
@@ -9110,7 +9110,7 @@
         </is>
       </c>
       <c r="F218" t="n">
-        <v>50</v>
+        <v>2000</v>
       </c>
       <c r="G218" t="n">
         <v>4</v>
@@ -9149,7 +9149,7 @@
         </is>
       </c>
       <c r="F219" t="n">
-        <v>30</v>
+        <v>1200</v>
       </c>
       <c r="G219" t="n">
         <v>3</v>
@@ -9188,7 +9188,7 @@
         </is>
       </c>
       <c r="F220" t="n">
-        <v>39</v>
+        <v>1560</v>
       </c>
       <c r="G220" t="n">
         <v>2</v>
@@ -9227,7 +9227,7 @@
         </is>
       </c>
       <c r="F221" t="n">
-        <v>42</v>
+        <v>1680</v>
       </c>
       <c r="G221" t="n">
         <v>1</v>
@@ -9266,7 +9266,7 @@
         </is>
       </c>
       <c r="F222" t="n">
-        <v>59</v>
+        <v>2360</v>
       </c>
       <c r="G222" t="n">
         <v>3</v>
@@ -9305,7 +9305,7 @@
         </is>
       </c>
       <c r="F223" t="n">
-        <v>14</v>
+        <v>560</v>
       </c>
       <c r="G223" t="n">
         <v>4</v>
@@ -9344,7 +9344,7 @@
         </is>
       </c>
       <c r="F224" t="n">
-        <v>66</v>
+        <v>2640</v>
       </c>
       <c r="G224" t="n">
         <v>2</v>
@@ -9383,7 +9383,7 @@
         </is>
       </c>
       <c r="F225" t="n">
-        <v>39</v>
+        <v>1560</v>
       </c>
       <c r="G225" t="n">
         <v>3</v>
@@ -9422,7 +9422,7 @@
         </is>
       </c>
       <c r="F226" t="n">
-        <v>19</v>
+        <v>760</v>
       </c>
       <c r="G226" t="n">
         <v>4</v>
@@ -9461,7 +9461,7 @@
         </is>
       </c>
       <c r="F227" t="n">
-        <v>53</v>
+        <v>2120</v>
       </c>
       <c r="G227" t="n">
         <v>4</v>
@@ -9500,7 +9500,7 @@
         </is>
       </c>
       <c r="F228" t="n">
-        <v>89</v>
+        <v>3560</v>
       </c>
       <c r="G228" t="n">
         <v>5</v>
@@ -9539,7 +9539,7 @@
         </is>
       </c>
       <c r="F229" t="n">
-        <v>46</v>
+        <v>1840</v>
       </c>
       <c r="G229" t="n">
         <v>5</v>
@@ -9578,7 +9578,7 @@
         </is>
       </c>
       <c r="F230" t="n">
-        <v>89</v>
+        <v>3560</v>
       </c>
       <c r="G230" t="n">
         <v>8</v>
@@ -9617,7 +9617,7 @@
         </is>
       </c>
       <c r="F231" t="n">
-        <v>97</v>
+        <v>3880</v>
       </c>
       <c r="G231" t="n">
         <v>1</v>
@@ -9656,7 +9656,7 @@
         </is>
       </c>
       <c r="F232" t="n">
-        <v>51</v>
+        <v>2040</v>
       </c>
       <c r="G232" t="n">
         <v>6</v>
@@ -9695,7 +9695,7 @@
         </is>
       </c>
       <c r="F233" t="n">
-        <v>50</v>
+        <v>2000</v>
       </c>
       <c r="G233" t="n">
         <v>3</v>
@@ -9734,7 +9734,7 @@
         </is>
       </c>
       <c r="F234" t="n">
-        <v>76</v>
+        <v>3040</v>
       </c>
       <c r="G234" t="n">
         <v>4</v>
@@ -9773,7 +9773,7 @@
         </is>
       </c>
       <c r="F235" t="n">
-        <v>79</v>
+        <v>3160</v>
       </c>
       <c r="G235" t="n">
         <v>5</v>
@@ -9812,7 +9812,7 @@
         </is>
       </c>
       <c r="F236" t="n">
-        <v>52</v>
+        <v>2080</v>
       </c>
       <c r="G236" t="n">
         <v>7</v>
@@ -9851,7 +9851,7 @@
         </is>
       </c>
       <c r="F237" t="n">
-        <v>84</v>
+        <v>3360</v>
       </c>
       <c r="G237" t="n">
         <v>8</v>
@@ -9890,7 +9890,7 @@
         </is>
       </c>
       <c r="F238" t="n">
-        <v>71</v>
+        <v>2840</v>
       </c>
       <c r="G238" t="n">
         <v>4</v>
@@ -9929,7 +9929,7 @@
         </is>
       </c>
       <c r="F239" t="n">
-        <v>39</v>
+        <v>1560</v>
       </c>
       <c r="G239" t="n">
         <v>4</v>
@@ -9968,7 +9968,7 @@
         </is>
       </c>
       <c r="F240" t="n">
-        <v>52</v>
+        <v>2080</v>
       </c>
       <c r="G240" t="n">
         <v>3</v>
@@ -10007,7 +10007,7 @@
         </is>
       </c>
       <c r="F241" t="n">
-        <v>63</v>
+        <v>2520</v>
       </c>
       <c r="G241" t="n">
         <v>2</v>
@@ -10046,7 +10046,7 @@
         </is>
       </c>
       <c r="F242" t="n">
-        <v>14</v>
+        <v>560</v>
       </c>
       <c r="G242" t="n">
         <v>1</v>
@@ -10085,7 +10085,7 @@
         </is>
       </c>
       <c r="F243" t="n">
-        <v>28</v>
+        <v>1120</v>
       </c>
       <c r="G243" t="n">
         <v>1</v>
@@ -10124,7 +10124,7 @@
         </is>
       </c>
       <c r="F244" t="n">
-        <v>50</v>
+        <v>2000</v>
       </c>
       <c r="G244" t="n">
         <v>5</v>
@@ -10163,7 +10163,7 @@
         </is>
       </c>
       <c r="F245" t="n">
-        <v>133</v>
+        <v>5320</v>
       </c>
       <c r="G245" t="n">
         <v>8</v>
@@ -10202,7 +10202,7 @@
         </is>
       </c>
       <c r="F246" t="n">
-        <v>30</v>
+        <v>1200</v>
       </c>
       <c r="G246" t="n">
         <v>4</v>
@@ -10241,7 +10241,7 @@
         </is>
       </c>
       <c r="F247" t="n">
-        <v>21</v>
+        <v>840</v>
       </c>
       <c r="G247" t="n">
         <v>3</v>
@@ -10280,7 +10280,7 @@
         </is>
       </c>
       <c r="F248" t="n">
-        <v>51</v>
+        <v>2040</v>
       </c>
       <c r="G248" t="n">
         <v>2</v>
@@ -10319,7 +10319,7 @@
         </is>
       </c>
       <c r="F249" t="n">
-        <v>102</v>
+        <v>4080</v>
       </c>
       <c r="G249" t="n">
         <v>5</v>
@@ -10358,7 +10358,7 @@
         </is>
       </c>
       <c r="F250" t="n">
-        <v>72</v>
+        <v>2880</v>
       </c>
       <c r="G250" t="n">
         <v>3</v>
@@ -10397,7 +10397,7 @@
         </is>
       </c>
       <c r="F251" t="n">
-        <v>79</v>
+        <v>3160</v>
       </c>
       <c r="G251" t="n">
         <v>4</v>
@@ -10436,7 +10436,7 @@
         </is>
       </c>
       <c r="F252" t="n">
-        <v>51</v>
+        <v>2040</v>
       </c>
       <c r="G252" t="n">
         <v>5</v>
@@ -10475,7 +10475,7 @@
         </is>
       </c>
       <c r="F253" t="n">
-        <v>13</v>
+        <v>520</v>
       </c>
       <c r="G253" t="n">
         <v>2</v>
@@ -10514,7 +10514,7 @@
         </is>
       </c>
       <c r="F254" t="n">
-        <v>34</v>
+        <v>1360</v>
       </c>
       <c r="G254" t="n">
         <v>1</v>
@@ -10553,7 +10553,7 @@
         </is>
       </c>
       <c r="F255" t="n">
-        <v>26</v>
+        <v>1040</v>
       </c>
       <c r="G255" t="n">
         <v>2</v>
@@ -10592,7 +10592,7 @@
         </is>
       </c>
       <c r="F256" t="n">
-        <v>94</v>
+        <v>3760</v>
       </c>
       <c r="G256" t="n">
         <v>6</v>
@@ -10631,7 +10631,7 @@
         </is>
       </c>
       <c r="F257" t="n">
-        <v>50</v>
+        <v>2000</v>
       </c>
       <c r="G257" t="n">
         <v>6</v>
@@ -10670,7 +10670,7 @@
         </is>
       </c>
       <c r="F258" t="n">
-        <v>81</v>
+        <v>3240</v>
       </c>
       <c r="G258" t="n">
         <v>6</v>
@@ -10709,7 +10709,7 @@
         </is>
       </c>
       <c r="F259" t="n">
-        <v>66</v>
+        <v>2640</v>
       </c>
       <c r="G259" t="n">
         <v>9</v>
@@ -10748,7 +10748,7 @@
         </is>
       </c>
       <c r="F260" t="n">
-        <v>55</v>
+        <v>2200</v>
       </c>
       <c r="G260" t="n">
         <v>3</v>
@@ -10787,7 +10787,7 @@
         </is>
       </c>
       <c r="F261" t="n">
-        <v>48</v>
+        <v>1920</v>
       </c>
       <c r="G261" t="n">
         <v>5</v>
@@ -10826,7 +10826,7 @@
         </is>
       </c>
       <c r="F262" t="n">
-        <v>20</v>
+        <v>800</v>
       </c>
       <c r="G262" t="n">
         <v>3</v>
@@ -10865,7 +10865,7 @@
         </is>
       </c>
       <c r="F263" t="n">
-        <v>33</v>
+        <v>1320</v>
       </c>
       <c r="H263" t="n">
         <v>8</v>
@@ -10901,7 +10901,7 @@
         </is>
       </c>
       <c r="F264" t="n">
-        <v>32</v>
+        <v>1280</v>
       </c>
       <c r="G264" t="n">
         <v>3</v>
@@ -10940,7 +10940,7 @@
         </is>
       </c>
       <c r="F265" t="n">
-        <v>36</v>
+        <v>1440</v>
       </c>
       <c r="G265" t="n">
         <v>5</v>
@@ -10979,7 +10979,7 @@
         </is>
       </c>
       <c r="F266" t="n">
-        <v>8</v>
+        <v>320</v>
       </c>
       <c r="G266" t="n">
         <v>2</v>
@@ -11018,7 +11018,7 @@
         </is>
       </c>
       <c r="F267" t="n">
-        <v>65</v>
+        <v>2600</v>
       </c>
       <c r="G267" t="n">
         <v>3</v>
@@ -11093,7 +11093,7 @@
         </is>
       </c>
       <c r="F269" t="n">
-        <v>32</v>
+        <v>1280</v>
       </c>
       <c r="G269" t="n">
         <v>1</v>
@@ -11132,7 +11132,7 @@
         </is>
       </c>
       <c r="F270" t="n">
-        <v>88</v>
+        <v>3520</v>
       </c>
       <c r="G270" t="n">
         <v>7</v>
@@ -11171,7 +11171,7 @@
         </is>
       </c>
       <c r="F271" t="n">
-        <v>16</v>
+        <v>640</v>
       </c>
       <c r="G271" t="n">
         <v>4</v>
@@ -11210,7 +11210,7 @@
         </is>
       </c>
       <c r="F272" t="n">
-        <v>50</v>
+        <v>2000</v>
       </c>
       <c r="G272" t="n">
         <v>5</v>
@@ -11249,7 +11249,7 @@
         </is>
       </c>
       <c r="F273" t="n">
-        <v>38</v>
+        <v>1520</v>
       </c>
       <c r="G273" t="n">
         <v>1</v>
@@ -11288,7 +11288,7 @@
         </is>
       </c>
       <c r="F274" t="n">
-        <v>51</v>
+        <v>2040</v>
       </c>
       <c r="G274" t="n">
         <v>8</v>
@@ -11327,7 +11327,7 @@
         </is>
       </c>
       <c r="F275" t="n">
-        <v>27</v>
+        <v>1080</v>
       </c>
       <c r="G275" t="n">
         <v>1</v>
@@ -11366,7 +11366,7 @@
         </is>
       </c>
       <c r="F276" t="n">
-        <v>18</v>
+        <v>720</v>
       </c>
       <c r="G276" t="n">
         <v>4</v>
@@ -11405,7 +11405,7 @@
         </is>
       </c>
       <c r="F277" t="n">
-        <v>53</v>
+        <v>2120</v>
       </c>
       <c r="G277" t="n">
         <v>3</v>
@@ -11444,7 +11444,7 @@
         </is>
       </c>
       <c r="F278" t="n">
-        <v>68</v>
+        <v>2720</v>
       </c>
       <c r="G278" t="n">
         <v>4</v>
@@ -11483,7 +11483,7 @@
         </is>
       </c>
       <c r="F279" t="n">
-        <v>38</v>
+        <v>1520</v>
       </c>
       <c r="G279" t="n">
         <v>4</v>
@@ -11522,7 +11522,7 @@
         </is>
       </c>
       <c r="F280" t="n">
-        <v>73</v>
+        <v>2920</v>
       </c>
       <c r="G280" t="n">
         <v>7</v>
@@ -11561,7 +11561,7 @@
         </is>
       </c>
       <c r="F281" t="n">
-        <v>43</v>
+        <v>1720</v>
       </c>
       <c r="G281" t="n">
         <v>2</v>
@@ -11600,7 +11600,7 @@
         </is>
       </c>
       <c r="F282" t="n">
-        <v>20</v>
+        <v>800</v>
       </c>
       <c r="G282" t="n">
         <v>2</v>
@@ -11639,7 +11639,7 @@
         </is>
       </c>
       <c r="F283" t="n">
-        <v>85</v>
+        <v>3400</v>
       </c>
       <c r="G283" t="n">
         <v>7</v>
@@ -11678,7 +11678,7 @@
         </is>
       </c>
       <c r="F284" t="n">
-        <v>29</v>
+        <v>1160</v>
       </c>
       <c r="G284" t="n">
         <v>3</v>
@@ -11717,7 +11717,7 @@
         </is>
       </c>
       <c r="F285" t="n">
-        <v>41</v>
+        <v>1640</v>
       </c>
       <c r="G285" t="n">
         <v>4</v>
@@ -11756,7 +11756,7 @@
         </is>
       </c>
       <c r="F286" t="n">
-        <v>37</v>
+        <v>1480</v>
       </c>
       <c r="G286" t="n">
         <v>3</v>
@@ -11795,7 +11795,7 @@
         </is>
       </c>
       <c r="F287" t="n">
-        <v>54</v>
+        <v>2160</v>
       </c>
       <c r="G287" t="n">
         <v>3</v>
@@ -11834,7 +11834,7 @@
         </is>
       </c>
       <c r="F288" t="n">
-        <v>60</v>
+        <v>2400</v>
       </c>
       <c r="G288" t="n">
         <v>5</v>
@@ -11873,7 +11873,7 @@
         </is>
       </c>
       <c r="F289" t="n">
-        <v>58</v>
+        <v>2320</v>
       </c>
       <c r="G289" t="n">
         <v>4</v>
@@ -11912,7 +11912,7 @@
         </is>
       </c>
       <c r="F290" t="n">
-        <v>52</v>
+        <v>2080</v>
       </c>
       <c r="G290" t="n">
         <v>5</v>
@@ -11951,7 +11951,7 @@
         </is>
       </c>
       <c r="F291" t="n">
-        <v>102</v>
+        <v>4080</v>
       </c>
       <c r="G291" t="n">
         <v>7</v>
@@ -11990,7 +11990,7 @@
         </is>
       </c>
       <c r="F292" t="n">
-        <v>42</v>
+        <v>1680</v>
       </c>
       <c r="G292" t="n">
         <v>4</v>
@@ -12029,7 +12029,7 @@
         </is>
       </c>
       <c r="F293" t="n">
-        <v>76</v>
+        <v>3040</v>
       </c>
       <c r="G293" t="n">
         <v>5</v>
@@ -12068,7 +12068,7 @@
         </is>
       </c>
       <c r="F294" t="n">
-        <v>27</v>
+        <v>1080</v>
       </c>
       <c r="G294" t="n">
         <v>3</v>
@@ -12107,7 +12107,7 @@
         </is>
       </c>
       <c r="F295" t="n">
-        <v>64</v>
+        <v>2560</v>
       </c>
       <c r="G295" t="n">
         <v>7</v>
@@ -12146,7 +12146,7 @@
         </is>
       </c>
       <c r="F296" t="n">
-        <v>23</v>
+        <v>920</v>
       </c>
       <c r="G296" t="n">
         <v>1</v>
@@ -12185,7 +12185,7 @@
         </is>
       </c>
       <c r="F297" t="n">
-        <v>85</v>
+        <v>3400</v>
       </c>
       <c r="G297" t="n">
         <v>6</v>
@@ -12224,7 +12224,7 @@
         </is>
       </c>
       <c r="F298" t="n">
-        <v>27</v>
+        <v>1080</v>
       </c>
       <c r="G298" t="n">
         <v>3</v>
@@ -12263,7 +12263,7 @@
         </is>
       </c>
       <c r="F299" t="n">
-        <v>49</v>
+        <v>1960</v>
       </c>
       <c r="G299" t="n">
         <v>5</v>
@@ -12302,7 +12302,7 @@
         </is>
       </c>
       <c r="F300" t="n">
-        <v>5</v>
+        <v>200</v>
       </c>
       <c r="G300" t="n">
         <v>2</v>
@@ -12341,7 +12341,7 @@
         </is>
       </c>
       <c r="F301" t="n">
-        <v>75</v>
+        <v>3000</v>
       </c>
       <c r="G301" t="n">
         <v>3</v>
@@ -12380,7 +12380,7 @@
         </is>
       </c>
       <c r="F302" t="n">
-        <v>18</v>
+        <v>720</v>
       </c>
       <c r="G302" t="n">
         <v>4</v>
@@ -12419,7 +12419,7 @@
         </is>
       </c>
       <c r="F303" t="n">
-        <v>88</v>
+        <v>3520</v>
       </c>
       <c r="G303" t="n">
         <v>7</v>
@@ -12458,7 +12458,7 @@
         </is>
       </c>
       <c r="F304" t="n">
-        <v>34</v>
+        <v>1360</v>
       </c>
       <c r="G304" t="n">
         <v>4</v>
@@ -12497,7 +12497,7 @@
         </is>
       </c>
       <c r="F305" t="n">
-        <v>28</v>
+        <v>1120</v>
       </c>
       <c r="G305" t="n">
         <v>2</v>
@@ -12536,7 +12536,7 @@
         </is>
       </c>
       <c r="F306" t="n">
-        <v>64</v>
+        <v>2560</v>
       </c>
       <c r="G306" t="n">
         <v>5</v>
@@ -12575,7 +12575,7 @@
         </is>
       </c>
       <c r="F307" t="n">
-        <v>53</v>
+        <v>2120</v>
       </c>
       <c r="G307" t="n">
         <v>2</v>
@@ -12614,7 +12614,7 @@
         </is>
       </c>
       <c r="F308" t="n">
-        <v>5</v>
+        <v>200</v>
       </c>
       <c r="G308" t="n">
         <v>3</v>
@@ -12653,7 +12653,7 @@
         </is>
       </c>
       <c r="F309" t="n">
-        <v>36</v>
+        <v>1440</v>
       </c>
       <c r="G309" t="n">
         <v>3</v>
@@ -12692,7 +12692,7 @@
         </is>
       </c>
       <c r="F310" t="n">
-        <v>39</v>
+        <v>1560</v>
       </c>
       <c r="G310" t="n">
         <v>2</v>
@@ -12731,7 +12731,7 @@
         </is>
       </c>
       <c r="F311" t="n">
-        <v>76</v>
+        <v>3040</v>
       </c>
       <c r="G311" t="n">
         <v>7</v>
@@ -12770,7 +12770,7 @@
         </is>
       </c>
       <c r="F312" t="n">
-        <v>27</v>
+        <v>1080</v>
       </c>
       <c r="G312" t="n">
         <v>1</v>
@@ -12809,7 +12809,7 @@
         </is>
       </c>
       <c r="F313" t="n">
-        <v>62</v>
+        <v>2480</v>
       </c>
       <c r="G313" t="n">
         <v>7</v>
@@ -12848,7 +12848,7 @@
         </is>
       </c>
       <c r="F314" t="n">
-        <v>115</v>
+        <v>4600</v>
       </c>
       <c r="G314" t="n">
         <v>7</v>
@@ -12887,7 +12887,7 @@
         </is>
       </c>
       <c r="F315" t="n">
-        <v>7</v>
+        <v>280</v>
       </c>
       <c r="G315" t="n">
         <v>5</v>
@@ -12926,7 +12926,7 @@
         </is>
       </c>
       <c r="F316" t="n">
-        <v>5</v>
+        <v>200</v>
       </c>
       <c r="G316" t="n">
         <v>5</v>
@@ -12965,7 +12965,7 @@
         </is>
       </c>
       <c r="F317" t="n">
-        <v>16</v>
+        <v>640</v>
       </c>
       <c r="G317" t="n">
         <v>1</v>
@@ -13004,7 +13004,7 @@
         </is>
       </c>
       <c r="F318" t="n">
-        <v>70</v>
+        <v>2800</v>
       </c>
       <c r="G318" t="n">
         <v>5</v>
@@ -13040,7 +13040,7 @@
         </is>
       </c>
       <c r="F319" t="n">
-        <v>27</v>
+        <v>1080</v>
       </c>
       <c r="G319" t="n">
         <v>6</v>
@@ -13079,7 +13079,7 @@
         </is>
       </c>
       <c r="F320" t="n">
-        <v>86</v>
+        <v>3440</v>
       </c>
       <c r="G320" t="n">
         <v>4</v>
@@ -13118,7 +13118,7 @@
         </is>
       </c>
       <c r="F321" t="n">
-        <v>55</v>
+        <v>2200</v>
       </c>
       <c r="G321" t="n">
         <v>4</v>
@@ -13157,7 +13157,7 @@
         </is>
       </c>
       <c r="F322" t="n">
-        <v>118</v>
+        <v>4720</v>
       </c>
       <c r="G322" t="n">
         <v>6</v>
@@ -13196,7 +13196,7 @@
         </is>
       </c>
       <c r="F323" t="n">
-        <v>125</v>
+        <v>5000</v>
       </c>
       <c r="G323" t="n">
         <v>6</v>
@@ -13235,7 +13235,7 @@
         </is>
       </c>
       <c r="F324" t="n">
-        <v>68</v>
+        <v>2720</v>
       </c>
       <c r="G324" t="n">
         <v>3</v>
@@ -13274,7 +13274,7 @@
         </is>
       </c>
       <c r="F325" t="n">
-        <v>41</v>
+        <v>1640</v>
       </c>
       <c r="G325" t="n">
         <v>7</v>
@@ -13313,7 +13313,7 @@
         </is>
       </c>
       <c r="F326" t="n">
-        <v>41</v>
+        <v>1640</v>
       </c>
       <c r="G326" t="n">
         <v>5</v>
@@ -13352,7 +13352,7 @@
         </is>
       </c>
       <c r="F327" t="n">
-        <v>15</v>
+        <v>600</v>
       </c>
       <c r="G327" t="n">
         <v>4</v>
@@ -13391,7 +13391,7 @@
         </is>
       </c>
       <c r="F328" t="n">
-        <v>39</v>
+        <v>1560</v>
       </c>
       <c r="G328" t="n">
         <v>2</v>
@@ -13430,7 +13430,7 @@
         </is>
       </c>
       <c r="F329" t="n">
-        <v>23</v>
+        <v>920</v>
       </c>
       <c r="G329" t="n">
         <v>1</v>
@@ -13469,7 +13469,7 @@
         </is>
       </c>
       <c r="F330" t="n">
-        <v>59</v>
+        <v>2360</v>
       </c>
       <c r="G330" t="n">
         <v>4</v>
@@ -13508,7 +13508,7 @@
         </is>
       </c>
       <c r="F331" t="n">
-        <v>95</v>
+        <v>3800</v>
       </c>
       <c r="G331" t="n">
         <v>6</v>
@@ -13547,7 +13547,7 @@
         </is>
       </c>
       <c r="F332" t="n">
-        <v>55</v>
+        <v>2200</v>
       </c>
       <c r="G332" t="n">
         <v>2</v>
@@ -13586,7 +13586,7 @@
         </is>
       </c>
       <c r="F333" t="n">
-        <v>18</v>
+        <v>720</v>
       </c>
       <c r="G333" t="n">
         <v>1</v>
@@ -13625,7 +13625,7 @@
         </is>
       </c>
       <c r="F334" t="n">
-        <v>53</v>
+        <v>2120</v>
       </c>
       <c r="G334" t="n">
         <v>5</v>
@@ -13664,7 +13664,7 @@
         </is>
       </c>
       <c r="F335" t="n">
-        <v>17</v>
+        <v>680</v>
       </c>
       <c r="G335" t="n">
         <v>3</v>
@@ -13703,7 +13703,7 @@
         </is>
       </c>
       <c r="F336" t="n">
-        <v>46</v>
+        <v>1840</v>
       </c>
       <c r="G336" t="n">
         <v>5</v>
@@ -13742,7 +13742,7 @@
         </is>
       </c>
       <c r="F337" t="n">
-        <v>54</v>
+        <v>2160</v>
       </c>
       <c r="G337" t="n">
         <v>6</v>
@@ -13781,7 +13781,7 @@
         </is>
       </c>
       <c r="F338" t="n">
-        <v>27</v>
+        <v>1080</v>
       </c>
       <c r="G338" t="n">
         <v>4</v>
@@ -13820,7 +13820,7 @@
         </is>
       </c>
       <c r="F339" t="n">
-        <v>33</v>
+        <v>1320</v>
       </c>
       <c r="G339" t="n">
         <v>2</v>
@@ -13859,7 +13859,7 @@
         </is>
       </c>
       <c r="F340" t="n">
-        <v>12</v>
+        <v>480</v>
       </c>
       <c r="G340" t="n">
         <v>2</v>
@@ -13898,7 +13898,7 @@
         </is>
       </c>
       <c r="F341" t="n">
-        <v>18</v>
+        <v>720</v>
       </c>
       <c r="G341" t="n">
         <v>5</v>
@@ -13937,7 +13937,7 @@
         </is>
       </c>
       <c r="F342" t="n">
-        <v>35</v>
+        <v>1400</v>
       </c>
       <c r="G342" t="n">
         <v>3</v>
@@ -13976,7 +13976,7 @@
         </is>
       </c>
       <c r="F343" t="n">
-        <v>58</v>
+        <v>2320</v>
       </c>
       <c r="G343" t="n">
         <v>4</v>
@@ -14015,7 +14015,7 @@
         </is>
       </c>
       <c r="F344" t="n">
-        <v>39</v>
+        <v>1560</v>
       </c>
       <c r="G344" t="n">
         <v>4</v>
@@ -14054,7 +14054,7 @@
         </is>
       </c>
       <c r="F345" t="n">
-        <v>5</v>
+        <v>200</v>
       </c>
       <c r="G345" t="n">
         <v>1</v>
@@ -14093,7 +14093,7 @@
         </is>
       </c>
       <c r="F346" t="n">
-        <v>94</v>
+        <v>3760</v>
       </c>
       <c r="G346" t="n">
         <v>5</v>
@@ -14132,7 +14132,7 @@
         </is>
       </c>
       <c r="F347" t="n">
-        <v>5</v>
+        <v>200</v>
       </c>
       <c r="G347" t="n">
         <v>4</v>
@@ -14171,7 +14171,7 @@
         </is>
       </c>
       <c r="F348" t="n">
-        <v>38</v>
+        <v>1520</v>
       </c>
       <c r="G348" t="n">
         <v>3</v>
@@ -14210,7 +14210,7 @@
         </is>
       </c>
       <c r="F349" t="n">
-        <v>83</v>
+        <v>3320</v>
       </c>
       <c r="G349" t="n">
         <v>5</v>
@@ -14249,7 +14249,7 @@
         </is>
       </c>
       <c r="F350" t="n">
-        <v>119</v>
+        <v>4760</v>
       </c>
       <c r="G350" t="n">
         <v>9</v>
@@ -14288,7 +14288,7 @@
         </is>
       </c>
       <c r="F351" t="n">
-        <v>99</v>
+        <v>3960</v>
       </c>
       <c r="G351" t="n">
         <v>6</v>
@@ -14327,7 +14327,7 @@
         </is>
       </c>
       <c r="F352" t="n">
-        <v>59</v>
+        <v>2360</v>
       </c>
       <c r="G352" t="n">
         <v>1</v>
@@ -14366,7 +14366,7 @@
         </is>
       </c>
       <c r="F353" t="n">
-        <v>98</v>
+        <v>3920</v>
       </c>
       <c r="G353" t="n">
         <v>4</v>
@@ -14405,7 +14405,7 @@
         </is>
       </c>
       <c r="F354" t="n">
-        <v>55</v>
+        <v>2200</v>
       </c>
       <c r="G354" t="n">
         <v>4</v>
@@ -14444,7 +14444,7 @@
         </is>
       </c>
       <c r="F355" t="n">
-        <v>42</v>
+        <v>1680</v>
       </c>
       <c r="G355" t="n">
         <v>3</v>
@@ -14483,7 +14483,7 @@
         </is>
       </c>
       <c r="F356" t="n">
-        <v>23</v>
+        <v>920</v>
       </c>
       <c r="G356" t="n">
         <v>1</v>
@@ -14522,7 +14522,7 @@
         </is>
       </c>
       <c r="F357" t="n">
-        <v>71</v>
+        <v>2840</v>
       </c>
       <c r="G357" t="n">
         <v>8</v>
@@ -14561,7 +14561,7 @@
         </is>
       </c>
       <c r="F358" t="n">
-        <v>31</v>
+        <v>1240</v>
       </c>
       <c r="G358" t="n">
         <v>3</v>
@@ -14600,7 +14600,7 @@
         </is>
       </c>
       <c r="F359" t="n">
-        <v>38</v>
+        <v>1520</v>
       </c>
       <c r="G359" t="n">
         <v>1</v>
@@ -14639,7 +14639,7 @@
         </is>
       </c>
       <c r="F360" t="n">
-        <v>63</v>
+        <v>2520</v>
       </c>
       <c r="G360" t="n">
         <v>7</v>
@@ -14678,7 +14678,7 @@
         </is>
       </c>
       <c r="F361" t="n">
-        <v>86</v>
+        <v>3440</v>
       </c>
       <c r="G361" t="n">
         <v>7</v>
@@ -14717,7 +14717,7 @@
         </is>
       </c>
       <c r="F362" t="n">
-        <v>18</v>
+        <v>720</v>
       </c>
       <c r="H362" t="n">
         <v>3</v>
@@ -14753,7 +14753,7 @@
         </is>
       </c>
       <c r="F363" t="n">
-        <v>37</v>
+        <v>1480</v>
       </c>
       <c r="G363" t="n">
         <v>5</v>
@@ -14792,7 +14792,7 @@
         </is>
       </c>
       <c r="F364" t="n">
-        <v>37</v>
+        <v>1480</v>
       </c>
       <c r="G364" t="n">
         <v>3</v>
@@ -14831,7 +14831,7 @@
         </is>
       </c>
       <c r="F365" t="n">
-        <v>28</v>
+        <v>1120</v>
       </c>
       <c r="G365" t="n">
         <v>1</v>
@@ -14870,7 +14870,7 @@
         </is>
       </c>
       <c r="F366" t="n">
-        <v>10</v>
+        <v>400</v>
       </c>
       <c r="G366" t="n">
         <v>6</v>
@@ -14909,7 +14909,7 @@
         </is>
       </c>
       <c r="F367" t="n">
-        <v>96</v>
+        <v>3840</v>
       </c>
       <c r="G367" t="n">
         <v>6</v>
@@ -14948,7 +14948,7 @@
         </is>
       </c>
       <c r="F368" t="n">
-        <v>18</v>
+        <v>720</v>
       </c>
       <c r="G368" t="n">
         <v>5</v>
@@ -14987,7 +14987,7 @@
         </is>
       </c>
       <c r="F369" t="n">
-        <v>46</v>
+        <v>1840</v>
       </c>
       <c r="G369" t="n">
         <v>5</v>
@@ -15026,7 +15026,7 @@
         </is>
       </c>
       <c r="F370" t="n">
-        <v>60</v>
+        <v>2400</v>
       </c>
       <c r="G370" t="n">
         <v>5</v>
@@ -15065,7 +15065,7 @@
         </is>
       </c>
       <c r="F371" t="n">
-        <v>76</v>
+        <v>3040</v>
       </c>
       <c r="G371" t="n">
         <v>5</v>
@@ -15104,7 +15104,7 @@
         </is>
       </c>
       <c r="F372" t="n">
-        <v>63</v>
+        <v>2520</v>
       </c>
       <c r="G372" t="n">
         <v>8</v>
@@ -15143,7 +15143,7 @@
         </is>
       </c>
       <c r="F373" t="n">
-        <v>36</v>
+        <v>1440</v>
       </c>
       <c r="G373" t="n">
         <v>5</v>
@@ -15182,7 +15182,7 @@
         </is>
       </c>
       <c r="F374" t="n">
-        <v>47</v>
+        <v>1880</v>
       </c>
       <c r="G374" t="n">
         <v>3</v>
@@ -15221,7 +15221,7 @@
         </is>
       </c>
       <c r="F375" t="n">
-        <v>16</v>
+        <v>640</v>
       </c>
       <c r="G375" t="n">
         <v>1</v>
@@ -15260,7 +15260,7 @@
         </is>
       </c>
       <c r="F376" t="n">
-        <v>55</v>
+        <v>2200</v>
       </c>
       <c r="G376" t="n">
         <v>3</v>
@@ -15299,7 +15299,7 @@
         </is>
       </c>
       <c r="F377" t="n">
-        <v>26</v>
+        <v>1040</v>
       </c>
       <c r="G377" t="n">
         <v>2</v>
@@ -15338,7 +15338,7 @@
         </is>
       </c>
       <c r="F378" t="n">
-        <v>9</v>
+        <v>360</v>
       </c>
       <c r="G378" t="n">
         <v>5</v>
@@ -15377,7 +15377,7 @@
         </is>
       </c>
       <c r="F379" t="n">
-        <v>114</v>
+        <v>4560</v>
       </c>
       <c r="G379" t="n">
         <v>8</v>
@@ -15416,7 +15416,7 @@
         </is>
       </c>
       <c r="F380" t="n">
-        <v>53</v>
+        <v>2120</v>
       </c>
       <c r="G380" t="n">
         <v>4</v>
@@ -15455,7 +15455,7 @@
         </is>
       </c>
       <c r="F381" t="n">
-        <v>91</v>
+        <v>3640</v>
       </c>
       <c r="G381" t="n">
         <v>4</v>
@@ -15494,7 +15494,7 @@
         </is>
       </c>
       <c r="F382" t="n">
-        <v>80</v>
+        <v>3200</v>
       </c>
       <c r="G382" t="n">
         <v>7</v>
@@ -15533,7 +15533,7 @@
         </is>
       </c>
       <c r="F383" t="n">
-        <v>112</v>
+        <v>4480</v>
       </c>
       <c r="G383" t="n">
         <v>9</v>
@@ -15572,7 +15572,7 @@
         </is>
       </c>
       <c r="F384" t="n">
-        <v>59</v>
+        <v>2360</v>
       </c>
       <c r="G384" t="n">
         <v>6</v>
@@ -15611,7 +15611,7 @@
         </is>
       </c>
       <c r="F385" t="n">
-        <v>22</v>
+        <v>880</v>
       </c>
       <c r="G385" t="n">
         <v>4</v>
@@ -15650,7 +15650,7 @@
         </is>
       </c>
       <c r="F386" t="n">
-        <v>32</v>
+        <v>1280</v>
       </c>
       <c r="G386" t="n">
         <v>1</v>
@@ -15689,7 +15689,7 @@
         </is>
       </c>
       <c r="F387" t="n">
-        <v>101</v>
+        <v>4040</v>
       </c>
       <c r="G387" t="n">
         <v>7</v>
@@ -15728,7 +15728,7 @@
         </is>
       </c>
       <c r="F388" t="n">
-        <v>58</v>
+        <v>2320</v>
       </c>
       <c r="G388" t="n">
         <v>5</v>
@@ -15767,7 +15767,7 @@
         </is>
       </c>
       <c r="F389" t="n">
-        <v>79</v>
+        <v>3160</v>
       </c>
       <c r="G389" t="n">
         <v>5</v>
@@ -15806,7 +15806,7 @@
         </is>
       </c>
       <c r="F390" t="n">
-        <v>41</v>
+        <v>1640</v>
       </c>
       <c r="G390" t="n">
         <v>3</v>
@@ -15845,7 +15845,7 @@
         </is>
       </c>
       <c r="F391" t="n">
-        <v>58</v>
+        <v>2320</v>
       </c>
       <c r="G391" t="n">
         <v>8</v>
@@ -15884,7 +15884,7 @@
         </is>
       </c>
       <c r="F392" t="n">
-        <v>51</v>
+        <v>2040</v>
       </c>
       <c r="G392" t="n">
         <v>7</v>
@@ -15923,7 +15923,7 @@
         </is>
       </c>
       <c r="F393" t="n">
-        <v>31</v>
+        <v>1240</v>
       </c>
       <c r="G393" t="n">
         <v>6</v>
@@ -15962,7 +15962,7 @@
         </is>
       </c>
       <c r="F394" t="n">
-        <v>19</v>
+        <v>760</v>
       </c>
       <c r="G394" t="n">
         <v>2</v>
@@ -16001,7 +16001,7 @@
         </is>
       </c>
       <c r="F395" t="n">
-        <v>25</v>
+        <v>1000</v>
       </c>
       <c r="G395" t="n">
         <v>2</v>
@@ -16076,7 +16076,7 @@
         </is>
       </c>
       <c r="F397" t="n">
-        <v>5</v>
+        <v>200</v>
       </c>
       <c r="G397" t="n">
         <v>1</v>
@@ -16115,7 +16115,7 @@
         </is>
       </c>
       <c r="F398" t="n">
-        <v>51</v>
+        <v>2040</v>
       </c>
       <c r="G398" t="n">
         <v>2</v>
@@ -16154,7 +16154,7 @@
         </is>
       </c>
       <c r="F399" t="n">
-        <v>35</v>
+        <v>1400</v>
       </c>
       <c r="G399" t="n">
         <v>4</v>
@@ -16193,7 +16193,7 @@
         </is>
       </c>
       <c r="F400" t="n">
-        <v>90</v>
+        <v>3600</v>
       </c>
       <c r="G400" t="n">
         <v>8</v>
@@ -16232,7 +16232,7 @@
         </is>
       </c>
       <c r="F401" t="n">
-        <v>82</v>
+        <v>3280</v>
       </c>
       <c r="G401" t="n">
         <v>7</v>
@@ -16271,7 +16271,7 @@
         </is>
       </c>
       <c r="F402" t="n">
-        <v>32</v>
+        <v>1280</v>
       </c>
       <c r="G402" t="n">
         <v>2</v>
@@ -16310,7 +16310,7 @@
         </is>
       </c>
       <c r="F403" t="n">
-        <v>85</v>
+        <v>3400</v>
       </c>
       <c r="G403" t="n">
         <v>7</v>
@@ -16349,7 +16349,7 @@
         </is>
       </c>
       <c r="F404" t="n">
-        <v>32</v>
+        <v>1280</v>
       </c>
       <c r="G404" t="n">
         <v>3</v>
@@ -16388,7 +16388,7 @@
         </is>
       </c>
       <c r="F405" t="n">
-        <v>18</v>
+        <v>720</v>
       </c>
       <c r="G405" t="n">
         <v>3</v>
@@ -16427,7 +16427,7 @@
         </is>
       </c>
       <c r="F406" t="n">
-        <v>112</v>
+        <v>4480</v>
       </c>
       <c r="G406" t="n">
         <v>8</v>
@@ -16466,7 +16466,7 @@
         </is>
       </c>
       <c r="F407" t="n">
-        <v>83</v>
+        <v>3320</v>
       </c>
       <c r="G407" t="n">
         <v>2</v>
@@ -16505,7 +16505,7 @@
         </is>
       </c>
       <c r="F408" t="n">
-        <v>34</v>
+        <v>1360</v>
       </c>
       <c r="G408" t="n">
         <v>6</v>
@@ -16544,7 +16544,7 @@
         </is>
       </c>
       <c r="F409" t="n">
-        <v>43</v>
+        <v>1720</v>
       </c>
       <c r="G409" t="n">
         <v>3</v>
@@ -16583,7 +16583,7 @@
         </is>
       </c>
       <c r="F410" t="n">
-        <v>68</v>
+        <v>2720</v>
       </c>
       <c r="G410" t="n">
         <v>4</v>
@@ -16622,7 +16622,7 @@
         </is>
       </c>
       <c r="F411" t="n">
-        <v>109</v>
+        <v>4360</v>
       </c>
       <c r="G411" t="n">
         <v>5</v>
@@ -16661,7 +16661,7 @@
         </is>
       </c>
       <c r="F412" t="n">
-        <v>57</v>
+        <v>2280</v>
       </c>
       <c r="G412" t="n">
         <v>3</v>
@@ -16700,7 +16700,7 @@
         </is>
       </c>
       <c r="F413" t="n">
-        <v>14</v>
+        <v>560</v>
       </c>
       <c r="G413" t="n">
         <v>1</v>
@@ -16739,7 +16739,7 @@
         </is>
       </c>
       <c r="F414" t="n">
-        <v>46</v>
+        <v>1840</v>
       </c>
       <c r="G414" t="n">
         <v>2</v>
@@ -16778,7 +16778,7 @@
         </is>
       </c>
       <c r="F415" t="n">
-        <v>39</v>
+        <v>1560</v>
       </c>
       <c r="G415" t="n">
         <v>3</v>
@@ -16817,7 +16817,7 @@
         </is>
       </c>
       <c r="F416" t="n">
-        <v>78</v>
+        <v>3120</v>
       </c>
       <c r="G416" t="n">
         <v>6</v>
@@ -16856,7 +16856,7 @@
         </is>
       </c>
       <c r="F417" t="n">
-        <v>48</v>
+        <v>1920</v>
       </c>
       <c r="G417" t="n">
         <v>5</v>
@@ -16895,7 +16895,7 @@
         </is>
       </c>
       <c r="F418" t="n">
-        <v>43</v>
+        <v>1720</v>
       </c>
       <c r="G418" t="n">
         <v>1</v>
@@ -16934,7 +16934,7 @@
         </is>
       </c>
       <c r="F419" t="n">
-        <v>17</v>
+        <v>680</v>
       </c>
       <c r="G419" t="n">
         <v>5</v>
@@ -16973,7 +16973,7 @@
         </is>
       </c>
       <c r="F420" t="n">
-        <v>11</v>
+        <v>440</v>
       </c>
       <c r="G420" t="n">
         <v>4</v>
@@ -17012,7 +17012,7 @@
         </is>
       </c>
       <c r="F421" t="n">
-        <v>66</v>
+        <v>2640</v>
       </c>
       <c r="G421" t="n">
         <v>6</v>
@@ -17051,7 +17051,7 @@
         </is>
       </c>
       <c r="F422" t="n">
-        <v>25</v>
+        <v>1000</v>
       </c>
       <c r="G422" t="n">
         <v>5</v>
@@ -17087,7 +17087,7 @@
         </is>
       </c>
       <c r="F423" t="n">
-        <v>49</v>
+        <v>1960</v>
       </c>
       <c r="G423" t="n">
         <v>3</v>
@@ -17126,7 +17126,7 @@
         </is>
       </c>
       <c r="F424" t="n">
-        <v>99</v>
+        <v>3960</v>
       </c>
       <c r="G424" t="n">
         <v>6</v>
@@ -17165,7 +17165,7 @@
         </is>
       </c>
       <c r="F425" t="n">
-        <v>23</v>
+        <v>920</v>
       </c>
       <c r="G425" t="n">
         <v>1</v>
@@ -17204,7 +17204,7 @@
         </is>
       </c>
       <c r="F426" t="n">
-        <v>30</v>
+        <v>1200</v>
       </c>
       <c r="G426" t="n">
         <v>3</v>
@@ -17243,7 +17243,7 @@
         </is>
       </c>
       <c r="F427" t="n">
-        <v>103</v>
+        <v>4120</v>
       </c>
       <c r="G427" t="n">
         <v>7</v>
@@ -17282,7 +17282,7 @@
         </is>
       </c>
       <c r="F428" t="n">
-        <v>44</v>
+        <v>1760</v>
       </c>
       <c r="G428" t="n">
         <v>4</v>
@@ -17321,7 +17321,7 @@
         </is>
       </c>
       <c r="F429" t="n">
-        <v>56</v>
+        <v>2240</v>
       </c>
       <c r="G429" t="n">
         <v>3</v>
@@ -17360,7 +17360,7 @@
         </is>
       </c>
       <c r="F430" t="n">
-        <v>21</v>
+        <v>840</v>
       </c>
       <c r="G430" t="n">
         <v>2</v>
@@ -17399,7 +17399,7 @@
         </is>
       </c>
       <c r="F431" t="n">
-        <v>148</v>
+        <v>5920</v>
       </c>
       <c r="G431" t="n">
         <v>9</v>
@@ -17438,7 +17438,7 @@
         </is>
       </c>
       <c r="F432" t="n">
-        <v>16</v>
+        <v>640</v>
       </c>
       <c r="G432" t="n">
         <v>5</v>
@@ -17477,7 +17477,7 @@
         </is>
       </c>
       <c r="F433" t="n">
-        <v>70</v>
+        <v>2800</v>
       </c>
       <c r="G433" t="n">
         <v>5</v>
@@ -17516,7 +17516,7 @@
         </is>
       </c>
       <c r="F434" t="n">
-        <v>64</v>
+        <v>2560</v>
       </c>
       <c r="G434" t="n">
         <v>4</v>
@@ -17555,7 +17555,7 @@
         </is>
       </c>
       <c r="F435" t="n">
-        <v>32</v>
+        <v>1280</v>
       </c>
       <c r="G435" t="n">
         <v>3</v>
@@ -17594,7 +17594,7 @@
         </is>
       </c>
       <c r="F436" t="n">
-        <v>73</v>
+        <v>2920</v>
       </c>
       <c r="G436" t="n">
         <v>4</v>
@@ -17633,7 +17633,7 @@
         </is>
       </c>
       <c r="F437" t="n">
-        <v>17</v>
+        <v>680</v>
       </c>
       <c r="G437" t="n">
         <v>4</v>
@@ -17672,7 +17672,7 @@
         </is>
       </c>
       <c r="F438" t="n">
-        <v>60</v>
+        <v>2400</v>
       </c>
       <c r="G438" t="n">
         <v>7</v>
@@ -17747,7 +17747,7 @@
         </is>
       </c>
       <c r="F440" t="n">
-        <v>116</v>
+        <v>4640</v>
       </c>
       <c r="G440" t="n">
         <v>7</v>
@@ -17786,7 +17786,7 @@
         </is>
       </c>
       <c r="F441" t="n">
-        <v>84</v>
+        <v>3360</v>
       </c>
       <c r="G441" t="n">
         <v>4</v>
@@ -17825,7 +17825,7 @@
         </is>
       </c>
       <c r="F442" t="n">
-        <v>94</v>
+        <v>3760</v>
       </c>
       <c r="G442" t="n">
         <v>9</v>
@@ -17864,7 +17864,7 @@
         </is>
       </c>
       <c r="F443" t="n">
-        <v>64</v>
+        <v>2560</v>
       </c>
       <c r="G443" t="n">
         <v>6</v>
@@ -17903,7 +17903,7 @@
         </is>
       </c>
       <c r="F444" t="n">
-        <v>13</v>
+        <v>520</v>
       </c>
       <c r="G444" t="n">
         <v>2</v>
@@ -17942,7 +17942,7 @@
         </is>
       </c>
       <c r="F445" t="n">
-        <v>49</v>
+        <v>1960</v>
       </c>
       <c r="G445" t="n">
         <v>1</v>
@@ -17981,7 +17981,7 @@
         </is>
       </c>
       <c r="F446" t="n">
-        <v>31</v>
+        <v>1240</v>
       </c>
       <c r="G446" t="n">
         <v>2</v>
@@ -18020,7 +18020,7 @@
         </is>
       </c>
       <c r="F447" t="n">
-        <v>45</v>
+        <v>1800</v>
       </c>
       <c r="G447" t="n">
         <v>4</v>
@@ -18059,7 +18059,7 @@
         </is>
       </c>
       <c r="F448" t="n">
-        <v>41</v>
+        <v>1640</v>
       </c>
       <c r="G448" t="n">
         <v>3</v>
@@ -18098,7 +18098,7 @@
         </is>
       </c>
       <c r="F449" t="n">
-        <v>28</v>
+        <v>1120</v>
       </c>
       <c r="G449" t="n">
         <v>3</v>
@@ -18137,7 +18137,7 @@
         </is>
       </c>
       <c r="F450" t="n">
-        <v>40</v>
+        <v>1600</v>
       </c>
       <c r="G450" t="n">
         <v>3</v>
@@ -18176,7 +18176,7 @@
         </is>
       </c>
       <c r="F451" t="n">
-        <v>66</v>
+        <v>2640</v>
       </c>
       <c r="G451" t="n">
         <v>6</v>
@@ -18215,7 +18215,7 @@
         </is>
       </c>
       <c r="F452" t="n">
-        <v>75</v>
+        <v>3000</v>
       </c>
       <c r="G452" t="n">
         <v>6</v>
@@ -18254,7 +18254,7 @@
         </is>
       </c>
       <c r="F453" t="n">
-        <v>39</v>
+        <v>1560</v>
       </c>
       <c r="G453" t="n">
         <v>1</v>
@@ -18293,7 +18293,7 @@
         </is>
       </c>
       <c r="F454" t="n">
-        <v>72</v>
+        <v>2880</v>
       </c>
       <c r="G454" t="n">
         <v>3</v>
@@ -18332,7 +18332,7 @@
         </is>
       </c>
       <c r="F455" t="n">
-        <v>82</v>
+        <v>3280</v>
       </c>
       <c r="G455" t="n">
         <v>7</v>
@@ -18371,7 +18371,7 @@
         </is>
       </c>
       <c r="F456" t="n">
-        <v>16</v>
+        <v>640</v>
       </c>
       <c r="G456" t="n">
         <v>5</v>
@@ -18410,7 +18410,7 @@
         </is>
       </c>
       <c r="F457" t="n">
-        <v>26</v>
+        <v>1040</v>
       </c>
       <c r="G457" t="n">
         <v>2</v>
@@ -18449,7 +18449,7 @@
         </is>
       </c>
       <c r="F458" t="n">
-        <v>5</v>
+        <v>200</v>
       </c>
       <c r="G458" t="n">
         <v>1</v>
@@ -18488,7 +18488,7 @@
         </is>
       </c>
       <c r="F459" t="n">
-        <v>29</v>
+        <v>1160</v>
       </c>
       <c r="G459" t="n">
         <v>3</v>
@@ -18527,7 +18527,7 @@
         </is>
       </c>
       <c r="F460" t="n">
-        <v>34</v>
+        <v>1360</v>
       </c>
       <c r="G460" t="n">
         <v>3</v>
@@ -18566,7 +18566,7 @@
         </is>
       </c>
       <c r="F461" t="n">
-        <v>88</v>
+        <v>3520</v>
       </c>
       <c r="G461" t="n">
         <v>5</v>
@@ -18605,7 +18605,7 @@
         </is>
       </c>
       <c r="F462" t="n">
-        <v>35</v>
+        <v>1400</v>
       </c>
       <c r="G462" t="n">
         <v>4</v>
@@ -18644,7 +18644,7 @@
         </is>
       </c>
       <c r="F463" t="n">
-        <v>72</v>
+        <v>2880</v>
       </c>
       <c r="G463" t="n">
         <v>5</v>
@@ -18683,7 +18683,7 @@
         </is>
       </c>
       <c r="F464" t="n">
-        <v>11</v>
+        <v>440</v>
       </c>
       <c r="G464" t="n">
         <v>3</v>
@@ -18722,7 +18722,7 @@
         </is>
       </c>
       <c r="F465" t="n">
-        <v>89</v>
+        <v>3560</v>
       </c>
       <c r="G465" t="n">
         <v>8</v>
@@ -18761,7 +18761,7 @@
         </is>
       </c>
       <c r="F466" t="n">
-        <v>36</v>
+        <v>1440</v>
       </c>
       <c r="G466" t="n">
         <v>3</v>
@@ -18800,7 +18800,7 @@
         </is>
       </c>
       <c r="F467" t="n">
-        <v>85</v>
+        <v>3400</v>
       </c>
       <c r="G467" t="n">
         <v>7</v>
@@ -21292,7 +21292,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>precio_referencia_soles</t>
+          <t>costo_unitario_referencia_soles</t>
         </is>
       </c>
     </row>
@@ -21304,7 +21304,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Limpieza CIP de tanques</t>
+          <t>Yogurt bebible de fresa 1 L</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -21313,7 +21313,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>91.59</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="3">
@@ -21324,7 +21324,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Falla de motor eléctrico</t>
+          <t>Galletas de vainilla x6</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -21333,7 +21333,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>321.65</v>
+        <v>3.22</v>
       </c>
     </row>
     <row r="4">
@@ -21344,7 +21344,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Limpieza de faja transportadora</t>
+          <t>Fideos spaghetti 500 g</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -21353,7 +21353,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>91.66</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="5">
@@ -21364,7 +21364,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Falta de materia prima</t>
+          <t>Néctar de durazno 1 L</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -21373,7 +21373,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>252.86</v>
+        <v>2.53</v>
       </c>
     </row>
     <row r="6">
@@ -21384,7 +21384,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Corte de energía</t>
+          <t>Aceite vegetal 1 L</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -21393,7 +21393,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>320.36</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="7">
@@ -21404,7 +21404,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Rotura de faja</t>
+          <t>Detergente en polvo 1 kg</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -21413,7 +21413,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>389.87</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="8">
@@ -21424,7 +21424,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Desgaste de rodamientos</t>
+          <t>Gaseosa sabor naranja 500 ml</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -21433,7 +21433,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>378.08</v>
+        <v>3.78</v>
       </c>
     </row>
     <row r="9">
@@ -21444,7 +21444,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Calibración de balanza</t>
+          <t>Agua de mesa 625 ml</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -21453,7 +21453,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>150.61</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="10">
@@ -21464,7 +21464,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Falla de variador de frecuencia</t>
+          <t>Pan de molde blanco 600 g</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -21473,7 +21473,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>325.93</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="11">
@@ -21484,7 +21484,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Sanitización de línea</t>
+          <t>Leche evaporada 400 g</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -21493,7 +21493,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>90.55</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="12">
@@ -21504,7 +21504,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Falta de envases</t>
+          <t>Mermelada de fresa 320 g</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -21513,7 +21513,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>254.88</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="13">
@@ -21524,7 +21524,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Calibración de termocupla</t>
+          <t>Atún en conserva 170 g</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -21533,7 +21533,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>150.91</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="14">
@@ -21544,7 +21544,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Falla de cadena transmisora</t>
+          <t>Chocolate en barra 90 g</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -21553,7 +21553,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>377.79</v>
+        <v>3.78</v>
       </c>
     </row>
     <row r="15">
@@ -21564,7 +21564,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Falta de etiquetas</t>
+          <t>Harina preparada 1 kg</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -21573,7 +21573,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>262.03</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="16">
@@ -21584,7 +21584,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Limpieza de moldes</t>
+          <t>Jabón de tocador 90 g</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -21593,7 +21593,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>89.72</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="17">
@@ -21604,7 +21604,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Calibración de manómetro</t>
+          <t>Shampoo herbal 400 ml</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -21613,7 +21613,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>152.36</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="18">
@@ -21624,7 +21624,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Calibración de sensor de nivel</t>
+          <t>Arroz embolsado 5 kg</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -21633,7 +21633,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>147.56</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="19">
@@ -21644,7 +21644,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Limpieza de filtros</t>
+          <t>Azúcar rubia 1 kg</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -21653,7 +21653,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>87.3</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="20">
@@ -21664,7 +21664,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Ajuste de dosificadora</t>
+          <t>Café instantáneo 50 g</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -21673,7 +21673,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>148.77</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="21">
@@ -21684,7 +21684,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Calibración de caudalímetro</t>
+          <t>Avena precocida 900 g</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -21693,7 +21693,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>148.64</v>
+        <v>1.49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>